<commit_message>
upload DPE FU v3
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NES.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCB1912-7881-4458-8433-915AE26F4824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F505445-54C5-4687-9411-57BB16443895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_processing_elements!$A$1:$V$117</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="594">
   <si>
     <t>index</t>
   </si>
@@ -2095,6 +2108,9 @@
   </si>
   <si>
     <t>DM_medication</t>
+  </si>
+  <si>
+    <t>undetermined</t>
   </si>
 </sst>
 </file>
@@ -2490,7 +2506,7 @@
     <col min="16" max="16" width="24" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="46" customWidth="1"/>
-    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="16" customWidth="1"/>
     <col min="22" max="22" width="52" customWidth="1"/>
@@ -8502,16 +8518,16 @@
       <c r="Q114" s="2"/>
       <c r="R114" s="2"/>
       <c r="S114" s="2" t="s">
-        <v>90</v>
+        <v>593</v>
       </c>
       <c r="T114" s="2" t="s">
-        <v>91</v>
+        <v>593</v>
       </c>
       <c r="U114" s="2" t="s">
-        <v>90</v>
+        <v>593</v>
       </c>
       <c r="V114" s="2" t="s">
-        <v>90</v>
+        <v>593</v>
       </c>
     </row>
     <row r="115" spans="1:22" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
correct cancer type variables
there is an additional variable in the data that was not in the dd that specifies for each cancer type if yes the participant has it
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NES.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F505445-54C5-4687-9411-57BB16443895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E67410A-3A2F-49B3-9A81-20D6FEED5BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_processing_elements" sheetId="1" r:id="rId1"/>
@@ -1495,11 +1495,6 @@
 If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
   </si>
   <si>
-    <t>Cancer_FU;
-Cancer_age_bladder;
-Cancer_year_bladder</t>
-  </si>
-  <si>
     <t>Cancer;
 Age diagnosis;
 Year diagnosis</t>
@@ -1521,7 +1516,468 @@
 yyyy</t>
   </si>
   <si>
+    <t>dis_cancer_breast_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Breast</t>
+  </si>
+  <si>
+    <t>Ever had breast cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Breast);
+What year was the participant diagnosed with Cancer (Breast)</t>
+  </si>
+  <si>
+    <t>dis_cancer_cervix_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Cervix</t>
+  </si>
+  <si>
+    <t>Ever had cervical cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Cervical);
+What year was the participant diagnosed with Cancer (Cervical)</t>
+  </si>
+  <si>
+    <t>dis_cancer_colorectal_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Colorectal</t>
+  </si>
+  <si>
+    <t>Ever had colorectal cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Intestine);
+What year was the participant diagnosed with Cancer (Intestine)</t>
+  </si>
+  <si>
+    <t>dis_cancer_kidney_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Kidney</t>
+  </si>
+  <si>
+    <t>Ever had kidney cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_throat_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Throat (Larynx or Pharynx)</t>
+  </si>
+  <si>
+    <t>Ever had throat cancer (pharyngeal or laryngeal cancer)</t>
+  </si>
+  <si>
+    <t>dis_cancer_leukaemia_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Leukaemia</t>
+  </si>
+  <si>
+    <t>Ever had leukaemia</t>
+  </si>
+  <si>
+    <t>dis_cancer_lung_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Lung</t>
+  </si>
+  <si>
+    <t>Ever had lung cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Lung);
+What year was the participant diagnosed with Cancer (Lung)</t>
+  </si>
+  <si>
+    <t>dis_cancer_lymphoma_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Lymphoma</t>
+  </si>
+  <si>
+    <t>Ever had lymphoma</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Lymphatic);
+What year was the participant diagnosed with Cancer (Lymphatic)</t>
+  </si>
+  <si>
+    <t>dis_cancer_prostate_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Prostate</t>
+  </si>
+  <si>
+    <t>Ever had prostate cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Prostatic);
+What year was the participant diagnosed with Cancer (Prostatic)</t>
+  </si>
+  <si>
+    <t>dis_cancer_skin_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Skin</t>
+  </si>
+  <si>
+    <t>Ever had skin cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Skin);
+What year was the participant diagnosed with Cancer (Skin)</t>
+  </si>
+  <si>
+    <t>dis_cancer_stomach_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Stomach</t>
+  </si>
+  <si>
+    <t>Ever had stomach cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_testicle_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Testicle</t>
+  </si>
+  <si>
+    <t>Ever had testicular cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Testicle);
+What year was the participant diagnosed with Cancer (Testicle)</t>
+  </si>
+  <si>
+    <t>dis_cancer_uterus_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Uterus</t>
+  </si>
+  <si>
+    <t>Ever had uterine cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_brain_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Brain</t>
+  </si>
+  <si>
+    <t>Ever had brain cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_liver_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Liver</t>
+  </si>
+  <si>
+    <t>Ever had liver cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_ovary_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Ovary</t>
+  </si>
+  <si>
+    <t>Ever had ovarian cancer</t>
+  </si>
+  <si>
+    <t>dis_cancer_pancreas_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Pancreas</t>
+  </si>
+  <si>
+    <t>Ever had pancreatic cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Pancreatic);
+What year was the participant diagnosed with Cancer (Pancreatic)</t>
+  </si>
+  <si>
+    <t>dis_cancer_thyroid_ever</t>
+  </si>
+  <si>
+    <t>Cancer ever - Thyroid</t>
+  </si>
+  <si>
+    <t>Ever had thyroid cancer</t>
+  </si>
+  <si>
+    <t>Did the participant have a cancer diagnosis?;
+What age was the participant diagnosed with Cancer (Thyroid);
+What year was the participant diagnosed with Cancer (Thyroid)</t>
+  </si>
+  <si>
+    <t>dis_hypercholesterolemia_ever</t>
+  </si>
+  <si>
+    <t>Hypercholesterolemia ever</t>
+  </si>
+  <si>
+    <t>Ever had hypercholesterolemia</t>
+  </si>
+  <si>
+    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
+If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Have you ever had have any of the following conditions? Yes/No) or there is a response option for "None of the above" for a list including this condition, the harmonized values can be Yes/No. 
+If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
+  </si>
+  <si>
+    <t>Dyslipidemia_FU</t>
+  </si>
+  <si>
+    <t>Elevated cholesterol levels</t>
+  </si>
+  <si>
+    <t>Did the participant have elevated cholesterol levels?</t>
+  </si>
+  <si>
+    <t>dis_depression</t>
+  </si>
+  <si>
+    <t>Depression</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant currently has depression</t>
+  </si>
+  <si>
+    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
+If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you have any of the following conditions? Yes/No) or there is a response option for "None of the above" for a list including this condition, the harmonized values can be Yes/No. 
+If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
+  </si>
+  <si>
+    <t>Depression_FU</t>
+  </si>
+  <si>
+    <t>Did the participant have depression?</t>
+  </si>
+  <si>
+    <t>dis_alzheimers_dementia</t>
+  </si>
+  <si>
+    <t>Alzheimer's/dementia</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant has Alzheimer's or other dementia</t>
+  </si>
+  <si>
+    <t>Dementia_FU</t>
+  </si>
+  <si>
+    <t>Dementia/Alzheimer's</t>
+  </si>
+  <si>
+    <t>Did the participant have Dementia/Alzheimers?</t>
+  </si>
+  <si>
+    <t>med_lipid_lowering_curr</t>
+  </si>
+  <si>
+    <t>Current use of lipid-lowering medication</t>
+  </si>
+  <si>
+    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
+If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you currently take any medication? Yes/No) or there is a response option for "None of the above" for a list including this medication, the harmonized values can be Yes/No. 
+If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
+  </si>
+  <si>
+    <t>med_blood_pressure_curr</t>
+  </si>
+  <si>
+    <t>Current use of medication to manage blood pressure</t>
+  </si>
+  <si>
+    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
+If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you currently take any medication? If yes, specify...) or there is a response option for "None of the above" for a list including this medication, the harmonized values can be Yes/No. 
+If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
+  </si>
+  <si>
+    <t>med_diabetes_curr</t>
+  </si>
+  <si>
+    <t>Current use of medication for diabetes</t>
+  </si>
+  <si>
+    <t>cog_dep_cesd20</t>
+  </si>
+  <si>
+    <t>Center for Epidemiologic Studies Depression Scale (CES-D) 20-item score</t>
+  </si>
+  <si>
+    <t>Where possible, validate the calculation of the score. Allowed range is 0-60.</t>
+  </si>
+  <si>
+    <t>cog_dep_cesd10</t>
+  </si>
+  <si>
+    <t>Center for Epidemiologic Studies Depression Scale (CES-D) 10-item score</t>
+  </si>
+  <si>
+    <t>Where possible, validate the calculation of the score. Allowed range is 0-30.</t>
+  </si>
+  <si>
+    <t>cog_dep_malaise</t>
+  </si>
+  <si>
+    <t>Malaise Inventory 9-item score</t>
+  </si>
+  <si>
+    <t>Where possible, validate the calculation of the score. Allowed range is 0-9.</t>
+  </si>
+  <si>
+    <t>cog_dep_kessler</t>
+  </si>
+  <si>
+    <t>Kessler Psychological Distress Scale (K-10) score</t>
+  </si>
+  <si>
+    <t>Where possible, validate the calculation of the score. Allowed range is 10-50.</t>
+  </si>
+  <si>
+    <t>cog_dep_phq9</t>
+  </si>
+  <si>
+    <t>Patient Health Questionnaire-9 (PHQ-9) score</t>
+  </si>
+  <si>
+    <t>Where possible, validate the calculation of the score. Allowed range is 0-27.</t>
+  </si>
+  <si>
+    <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
+  </si>
+  <si>
+    <t>cog_mci_mmse</t>
+  </si>
+  <si>
+    <t>Mini-Mental State Examination (MMSE) score</t>
+  </si>
+  <si>
+    <t>cog_mci_moca</t>
+  </si>
+  <si>
+    <t>Montreal Cognitive Assessment (MoCA) score</t>
+  </si>
+  <si>
+    <t>dth_status</t>
+  </si>
+  <si>
+    <t>Death status</t>
+  </si>
+  <si>
+    <t>Indicator of whether the participant is deceased</t>
+  </si>
+  <si>
+    <t>dth_date_day</t>
+  </si>
+  <si>
+    <t>Death date - Day</t>
+  </si>
+  <si>
+    <t>dth_date_month</t>
+  </si>
+  <si>
+    <t>Death date - Month</t>
+  </si>
+  <si>
+    <t>dth_date_year</t>
+  </si>
+  <si>
+    <t>Death date - Year</t>
+  </si>
+  <si>
+    <t>Consumption frequency was not collected; only quantity (glasses per week) is available. Frequency could in principle be banded from quantity, but the "Monthly" category is unreachable from a weekly count</t>
+  </si>
+  <si>
+    <t>The follow-up questionnaire collected only the change in smoking behaviour over the past year (started / stopped / smoked less / no change), not current status. Categories 1, 2 and 3 imply current status, but the "No change" category does not, so status cannot be established from the follow-up</t>
+  </si>
+  <si>
+    <t>NES did not collect a distinct ischemic/coronary heart disease item. Derived as myocardial infarction or angina pectoris.</t>
+  </si>
+  <si>
     <t>case_when(
+MI_FU == 1 ~ 1L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>The study specific study variables includes Transiant Ischemic Attack (TIA)</t>
+  </si>
+  <si>
+    <t>case_when(
+Hypertension_FU == 1 | Hypertension_medication == 1 ~ 1L;
+Hypertension_FU == 0 &amp; Hypertension_medication == 0 ~ 0L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>Study specific variable only collects Type 1 and Type 2.</t>
+  </si>
+  <si>
+    <t>case_when(
+Dyslipidemia_medication == 1 | Dyslipidemia_statins == 1 | Dyslipidemia_medication_cholesterol_lowering == 1 ~ 1L;
+Dyslipidemia_medication == 0 ~ 0L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>Dyslipidemia_medication;
+Dyslipidemia_statins;
+Dyslipidemia_medication_cholesterol_lowering</t>
+  </si>
+  <si>
+    <t>Use medication;
+Which statine;
+Other cholesterol-lowering medication</t>
+  </si>
+  <si>
+    <t>Did the participant use medication?;
+Which Statine is the participant using;
+What other cholesterol-lowering medication did the participant take?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+NA</t>
+  </si>
+  <si>
+    <t>Did the participant use medication?</t>
+  </si>
+  <si>
+    <t>Use medication</t>
+  </si>
+  <si>
+    <t>Hypertension_medication</t>
+  </si>
+  <si>
+    <t>DM_medication</t>
+  </si>
+  <si>
+    <t>undetermined</t>
+  </si>
+  <si>
+    <t>Cancer_FU;
+Cancer_age_bladder;
+Cancer_year_bladder;
+Cancer_type_bladder</t>
+  </si>
+  <si>
+    <t>case_when(
+Cancer_type_bladder == 1 ~ 1L;
 !is.na(Cancer_age_bladder) &amp; Cancer_age_bladder != "." ~ 1L;
 !is.na(Cancer_year_bladder) &amp; Cancer_year_bladder != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1529,26 +1985,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_breast_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Breast</t>
-  </si>
-  <si>
-    <t>Ever had breast cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_breast;
-Cancer_year_breast</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Breast);
-What year was the participant diagnosed with Cancer (Breast)</t>
+Cancer_year_breast;
+Cancer_type_breast</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_breast == 1 ~ 1L;
 !is.na(Cancer_age_breast) &amp; Cancer_age_breast != "." ~ 1L;
 !is.na(Cancer_year_breast) &amp; Cancer_year_breast != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1556,26 +2000,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_cervix_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Cervix</t>
-  </si>
-  <si>
-    <t>Ever had cervical cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_cervical;
-Cancer_year_cervical</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Cervical);
-What year was the participant diagnosed with Cancer (Cervical)</t>
+Cancer_year_cervical;
+Cancer_type_cervical</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_cervical == 1 ~ 1L;
 !is.na(Cancer_age_cervical) &amp; Cancer_age_cervical != "." ~ 1L;
 !is.na(Cancer_year_cervical) &amp; Cancer_year_cervical != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1583,26 +2015,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_colorectal_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Colorectal</t>
-  </si>
-  <si>
-    <t>Ever had colorectal cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_intestinal;
-Cancer_year_intestinal</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Intestine);
-What year was the participant diagnosed with Cancer (Intestine)</t>
+Cancer_year_intestinal;
+Cancer_type_intestinal</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_intestinal == 1  ~ 1L;
 !is.na(Cancer_age_intestinal) &amp; Cancer_age_intestinal != "." ~ 1L;
 !is.na(Cancer_year_intestinal) &amp; Cancer_year_intestinal != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1610,53 +2030,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_kidney_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Kidney</t>
-  </si>
-  <si>
-    <t>Ever had kidney cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_throat_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Throat (Larynx or Pharynx)</t>
-  </si>
-  <si>
-    <t>Ever had throat cancer (pharyngeal or laryngeal cancer)</t>
-  </si>
-  <si>
-    <t>dis_cancer_leukaemia_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Leukaemia</t>
-  </si>
-  <si>
-    <t>Ever had leukaemia</t>
-  </si>
-  <si>
-    <t>dis_cancer_lung_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Lung</t>
-  </si>
-  <si>
-    <t>Ever had lung cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_lung;
-Cancer_year_lung</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Lung);
-What year was the participant diagnosed with Cancer (Lung)</t>
+Cancer_year_lung;
+Cancer_type_lung</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_lung == 1 ~ 1L;
 !is.na(Cancer_age_lung) &amp; Cancer_age_lung != "." ~ 1L;
 !is.na(Cancer_year_lung) &amp; Cancer_year_lung != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1664,26 +2045,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_lymphoma_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Lymphoma</t>
-  </si>
-  <si>
-    <t>Ever had lymphoma</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_lymphatic;
-Cancer_year_lymphatic</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Lymphatic);
-What year was the participant diagnosed with Cancer (Lymphatic)</t>
+Cancer_year_lymphatic;
+Cancer_type_lymphatic</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_lymphatic == 1 ~ 1L;
 !is.na(Cancer_age_lymphatic) &amp; Cancer_age_lymphatic != "." ~ 1L;
 !is.na(Cancer_year_lymphatic) &amp; Cancer_year_lymphatic != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1691,26 +2060,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_prostate_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Prostate</t>
-  </si>
-  <si>
-    <t>Ever had prostate cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_prostatic;
-Cancer_year_prostatic</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Prostatic);
-What year was the participant diagnosed with Cancer (Prostatic)</t>
+Cancer_year_prostatic;
+Cancer_type_prostatic</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_prostatic == 1 ~ 1L;
 !is.na(Cancer_age_prostatic) &amp; Cancer_age_prostatic != "." ~ 1L;
 !is.na(Cancer_year_prostatic) &amp; Cancer_year_prostatic != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1718,26 +2075,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_skin_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Skin</t>
-  </si>
-  <si>
-    <t>Ever had skin cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_skin;
-Cancer_year_skin</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Skin);
-What year was the participant diagnosed with Cancer (Skin)</t>
+Cancer_year_skin;
+Cancer_type_skin</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_skin == 1 ~ 1L;
 !is.na(Cancer_age_skin) &amp; Cancer_age_skin != "." ~ 1L;
 !is.na(Cancer_year_skin) &amp; Cancer_year_skin != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1745,35 +2090,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_stomach_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Stomach</t>
-  </si>
-  <si>
-    <t>Ever had stomach cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_testicle_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Testicle</t>
-  </si>
-  <si>
-    <t>Ever had testicular cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_testicle;
-Cancer_year_testicle</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Testicle);
-What year was the participant diagnosed with Cancer (Testicle)</t>
+Cancer_year_testicle;
+Cancer_type_testicle</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_testicle == 1 ~ 1L;
 !is.na(Cancer_age_testicle) &amp; Cancer_age_testicle != "." ~ 1L;
 !is.na(Cancer_year_testicle) &amp; Cancer_year_testicle != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1781,62 +2105,14 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_uterus_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Uterus</t>
-  </si>
-  <si>
-    <t>Ever had uterine cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_brain_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Brain</t>
-  </si>
-  <si>
-    <t>Ever had brain cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_liver_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Liver</t>
-  </si>
-  <si>
-    <t>Ever had liver cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_ovary_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Ovary</t>
-  </si>
-  <si>
-    <t>Ever had ovarian cancer</t>
-  </si>
-  <si>
-    <t>dis_cancer_pancreas_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Pancreas</t>
-  </si>
-  <si>
-    <t>Ever had pancreatic cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_pancreatic;
-Cancer_year_pancreatic</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Pancreatic);
-What year was the participant diagnosed with Cancer (Pancreatic)</t>
+Cancer_year_pancreatic;
+Cancer_type_pancreatic</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_pancreatic == 1 ~ 1L;
 !is.na(Cancer_age_pancreatic) &amp; Cancer_age_pancreatic != "." ~ 1L;
 !is.na(Cancer_year_pancreatic) &amp; Cancer_year_pancreatic != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
@@ -1844,273 +2120,19 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>dis_cancer_thyroid_ever</t>
-  </si>
-  <si>
-    <t>Cancer ever - Thyroid</t>
-  </si>
-  <si>
-    <t>Ever had thyroid cancer</t>
-  </si>
-  <si>
     <t>Cancer_FU;
 Cancer_age_thyroid;
-Cancer_year_thyroid</t>
-  </si>
-  <si>
-    <t>Did the participant have a cancer diagnosis?;
-What age was the participant diagnosed with Cancer (Thyroid);
-What year was the participant diagnosed with Cancer (Thyroid)</t>
+Cancer_year_thyroid;
+Cancer_type_thyroid</t>
   </si>
   <si>
     <t>case_when(
+Cancer_type_thyroid == 1 ~ 1L;
 !is.na(Cancer_age_thyroid) &amp; Cancer_age_thyroid != "." ~ 1L;
 !is.na(Cancer_year_thyroid) &amp; Cancer_year_thyroid != "." ~ 1L;
 Cancer_FU == 0 ~ 0L;
 Cancer_FU == 1 ~ 2L;
 ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>dis_hypercholesterolemia_ever</t>
-  </si>
-  <si>
-    <t>Hypercholesterolemia ever</t>
-  </si>
-  <si>
-    <t>Ever had hypercholesterolemia</t>
-  </si>
-  <si>
-    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
-If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Have you ever had have any of the following conditions? Yes/No) or there is a response option for "None of the above" for a list including this condition, the harmonized values can be Yes/No. 
-If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
-  </si>
-  <si>
-    <t>Dyslipidemia_FU</t>
-  </si>
-  <si>
-    <t>Elevated cholesterol levels</t>
-  </si>
-  <si>
-    <t>Did the participant have elevated cholesterol levels?</t>
-  </si>
-  <si>
-    <t>dis_depression</t>
-  </si>
-  <si>
-    <t>Depression</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant currently has depression</t>
-  </si>
-  <si>
-    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
-If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you have any of the following conditions? Yes/No) or there is a response option for "None of the above" for a list including this condition, the harmonized values can be Yes/No. 
-If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
-  </si>
-  <si>
-    <t>Depression_FU</t>
-  </si>
-  <si>
-    <t>Did the participant have depression?</t>
-  </si>
-  <si>
-    <t>dis_alzheimers_dementia</t>
-  </si>
-  <si>
-    <t>Alzheimer's/dementia</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant has Alzheimer's or other dementia</t>
-  </si>
-  <si>
-    <t>Dementia_FU</t>
-  </si>
-  <si>
-    <t>Dementia/Alzheimer's</t>
-  </si>
-  <si>
-    <t>Did the participant have Dementia/Alzheimers?</t>
-  </si>
-  <si>
-    <t>med_lipid_lowering_curr</t>
-  </si>
-  <si>
-    <t>Current use of lipid-lowering medication</t>
-  </si>
-  <si>
-    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
-If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you currently take any medication? Yes/No) or there is a response option for "None of the above" for a list including this medication, the harmonized values can be Yes/No. 
-If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
-  </si>
-  <si>
-    <t>med_blood_pressure_curr</t>
-  </si>
-  <si>
-    <t>Current use of medication to manage blood pressure</t>
-  </si>
-  <si>
-    <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
-If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Do you currently take any medication? If yes, specify...) or there is a response option for "None of the above" for a list including this medication, the harmonized values can be Yes/No. 
-If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
-  </si>
-  <si>
-    <t>med_diabetes_curr</t>
-  </si>
-  <si>
-    <t>Current use of medication for diabetes</t>
-  </si>
-  <si>
-    <t>cog_dep_cesd20</t>
-  </si>
-  <si>
-    <t>Center for Epidemiologic Studies Depression Scale (CES-D) 20-item score</t>
-  </si>
-  <si>
-    <t>Where possible, validate the calculation of the score. Allowed range is 0-60.</t>
-  </si>
-  <si>
-    <t>cog_dep_cesd10</t>
-  </si>
-  <si>
-    <t>Center for Epidemiologic Studies Depression Scale (CES-D) 10-item score</t>
-  </si>
-  <si>
-    <t>Where possible, validate the calculation of the score. Allowed range is 0-30.</t>
-  </si>
-  <si>
-    <t>cog_dep_malaise</t>
-  </si>
-  <si>
-    <t>Malaise Inventory 9-item score</t>
-  </si>
-  <si>
-    <t>Where possible, validate the calculation of the score. Allowed range is 0-9.</t>
-  </si>
-  <si>
-    <t>cog_dep_kessler</t>
-  </si>
-  <si>
-    <t>Kessler Psychological Distress Scale (K-10) score</t>
-  </si>
-  <si>
-    <t>Where possible, validate the calculation of the score. Allowed range is 10-50.</t>
-  </si>
-  <si>
-    <t>cog_dep_phq9</t>
-  </si>
-  <si>
-    <t>Patient Health Questionnaire-9 (PHQ-9) score</t>
-  </si>
-  <si>
-    <t>Where possible, validate the calculation of the score. Allowed range is 0-27.</t>
-  </si>
-  <si>
-    <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
-  </si>
-  <si>
-    <t>cog_mci_mmse</t>
-  </si>
-  <si>
-    <t>Mini-Mental State Examination (MMSE) score</t>
-  </si>
-  <si>
-    <t>cog_mci_moca</t>
-  </si>
-  <si>
-    <t>Montreal Cognitive Assessment (MoCA) score</t>
-  </si>
-  <si>
-    <t>dth_status</t>
-  </si>
-  <si>
-    <t>Death status</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is deceased</t>
-  </si>
-  <si>
-    <t>dth_date_day</t>
-  </si>
-  <si>
-    <t>Death date - Day</t>
-  </si>
-  <si>
-    <t>dth_date_month</t>
-  </si>
-  <si>
-    <t>Death date - Month</t>
-  </si>
-  <si>
-    <t>dth_date_year</t>
-  </si>
-  <si>
-    <t>Death date - Year</t>
-  </si>
-  <si>
-    <t>Consumption frequency was not collected; only quantity (glasses per week) is available. Frequency could in principle be banded from quantity, but the "Monthly" category is unreachable from a weekly count</t>
-  </si>
-  <si>
-    <t>The follow-up questionnaire collected only the change in smoking behaviour over the past year (started / stopped / smoked less / no change), not current status. Categories 1, 2 and 3 imply current status, but the "No change" category does not, so status cannot be established from the follow-up</t>
-  </si>
-  <si>
-    <t>NES did not collect a distinct ischemic/coronary heart disease item. Derived as myocardial infarction or angina pectoris.</t>
-  </si>
-  <si>
-    <t>case_when(
-MI_FU == 1 ~ 1L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>The study specific study variables includes Transiant Ischemic Attack (TIA)</t>
-  </si>
-  <si>
-    <t>case_when(
-Hypertension_FU == 1 | Hypertension_medication == 1 ~ 1L;
-Hypertension_FU == 0 &amp; Hypertension_medication == 0 ~ 0L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>Study specific variable only collects Type 1 and Type 2.</t>
-  </si>
-  <si>
-    <t>case_when(
-Dyslipidemia_medication == 1 | Dyslipidemia_statins == 1 | Dyslipidemia_medication_cholesterol_lowering == 1 ~ 1L;
-Dyslipidemia_medication == 0 ~ 0L;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>Dyslipidemia_medication;
-Dyslipidemia_statins;
-Dyslipidemia_medication_cholesterol_lowering</t>
-  </si>
-  <si>
-    <t>Use medication;
-Which statine;
-Other cholesterol-lowering medication</t>
-  </si>
-  <si>
-    <t>Did the participant use medication?;
-Which Statine is the participant using;
-What other cholesterol-lowering medication did the participant take?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-NA</t>
-  </si>
-  <si>
-    <t>Did the participant use medication?</t>
-  </si>
-  <si>
-    <t>Use medication</t>
-  </si>
-  <si>
-    <t>Hypertension_medication</t>
-  </si>
-  <si>
-    <t>DM_medication</t>
-  </si>
-  <si>
-    <t>undetermined</t>
   </si>
 </sst>
 </file>
@@ -2129,10 +2151,12 @@
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2488,7 +2512,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V117"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -2506,13 +2530,13 @@
     <col min="16" max="16" width="24" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="46" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" customWidth="1"/>
+    <col min="19" max="19" width="14.1796875" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="16" customWidth="1"/>
     <col min="22" max="22" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2580,7 +2604,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2636,7 +2660,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2684,7 +2708,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="213.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="210" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2732,7 +2756,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2780,7 +2804,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2840,7 +2864,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2896,7 +2920,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2956,7 +2980,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="128.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" ht="126" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3008,7 +3032,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3060,7 +3084,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="142.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" ht="140" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3110,7 +3134,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3162,7 +3186,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3210,7 +3234,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3256,7 +3280,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="114" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" ht="112" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3306,7 +3330,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3354,7 +3378,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3406,7 +3430,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3458,7 +3482,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3506,7 +3530,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3558,7 +3582,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3606,7 +3630,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3658,7 +3682,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3710,7 +3734,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3758,7 +3782,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3806,7 +3830,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3852,7 +3876,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3904,7 +3928,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -3956,7 +3980,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -4008,7 +4032,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -4060,7 +4084,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -4108,7 +4132,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -4156,7 +4180,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -4204,7 +4228,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -4252,7 +4276,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -4300,7 +4324,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -4348,7 +4372,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:22" ht="114" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:22" ht="98" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -4398,7 +4422,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -4446,7 +4470,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -4494,7 +4518,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4546,7 +4570,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4596,7 +4620,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4648,7 +4672,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4700,7 +4724,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -4748,7 +4772,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:22" ht="84" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -4808,7 +4832,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="46" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -4851,7 +4875,7 @@
         <v>31</v>
       </c>
       <c r="R46" s="2" t="s">
-        <v>577</v>
+        <v>555</v>
       </c>
       <c r="S46" s="2" t="s">
         <v>90</v>
@@ -4866,7 +4890,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:22" ht="99.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:22" ht="84" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -4913,7 +4937,7 @@
         <v>31</v>
       </c>
       <c r="R47" s="2" t="s">
-        <v>578</v>
+        <v>556</v>
       </c>
       <c r="S47" s="2" t="s">
         <v>90</v>
@@ -4928,7 +4952,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -4978,7 +5002,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -5030,7 +5054,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -5078,7 +5102,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="156.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:22" ht="154" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -5128,7 +5152,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -5178,7 +5202,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -5228,7 +5252,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -5276,7 +5300,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -5324,7 +5348,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="156.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:22" ht="154" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -5372,7 +5396,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -5422,7 +5446,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -5472,7 +5496,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -5522,7 +5546,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:22" ht="84" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -5570,7 +5594,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -5620,7 +5644,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:22" ht="84" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -5670,7 +5694,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="128.25" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:22" ht="112" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -5722,7 +5746,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -5772,7 +5796,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:22" ht="70" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -5824,7 +5848,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -5872,7 +5896,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -5920,7 +5944,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="68" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -5970,7 +5994,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="69" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:22" ht="392" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -6030,7 +6054,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="70" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -6077,7 +6101,7 @@
         <v>31</v>
       </c>
       <c r="R70" s="3" t="s">
-        <v>579</v>
+        <v>557</v>
       </c>
       <c r="S70" s="2" t="s">
         <v>32</v>
@@ -6089,10 +6113,10 @@
         <v>231</v>
       </c>
       <c r="V70" s="3" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="71" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -6152,7 +6176,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="72" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -6212,7 +6236,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="73" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -6259,7 +6283,7 @@
         <v>31</v>
       </c>
       <c r="R73" s="3" t="s">
-        <v>581</v>
+        <v>559</v>
       </c>
       <c r="S73" s="2" t="s">
         <v>32</v>
@@ -6274,7 +6298,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="74" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -6334,7 +6358,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="75" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -6394,7 +6418,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="76" spans="1:22" ht="399" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:22" ht="350" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -6456,7 +6480,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="77" spans="1:22" ht="285" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -6513,10 +6537,10 @@
         <v>231</v>
       </c>
       <c r="V77" s="3" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="78" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -6576,7 +6600,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="79" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -6638,7 +6662,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="80" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:22" ht="56" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -6683,7 +6707,7 @@
         <v>31</v>
       </c>
       <c r="R80" s="3" t="s">
-        <v>583</v>
+        <v>561</v>
       </c>
       <c r="S80" s="2" t="s">
         <v>32</v>
@@ -6698,7 +6722,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="1:22" ht="228" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:22" ht="196" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -6758,7 +6782,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -6788,19 +6812,19 @@
         <v>326</v>
       </c>
       <c r="M82" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="N82" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="N82" s="2" t="s">
+      <c r="O82" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="O82" s="2" t="s">
+      <c r="P82" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="P82" s="2" t="s">
+      <c r="Q82" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q82" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R82" s="2"/>
       <c r="S82" s="2" t="s">
@@ -6812,11 +6836,11 @@
       <c r="U82" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="V82" s="3" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="83" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+      <c r="V82" s="2" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -6824,13 +6848,13 @@
         <v>22</v>
       </c>
       <c r="C83" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="E83" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>50</v>
@@ -6846,19 +6870,19 @@
         <v>326</v>
       </c>
       <c r="M83" s="2" t="s">
-        <v>440</v>
+        <v>574</v>
       </c>
       <c r="N83" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O83" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="P83" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q83" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q83" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R83" s="2"/>
       <c r="S83" s="2" t="s">
@@ -6871,10 +6895,10 @@
         <v>231</v>
       </c>
       <c r="V83" s="2" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="84" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -6882,13 +6906,13 @@
         <v>22</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>50</v>
@@ -6904,19 +6928,19 @@
         <v>326</v>
       </c>
       <c r="M84" s="2" t="s">
-        <v>446</v>
+        <v>576</v>
       </c>
       <c r="N84" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O84" s="2" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="P84" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q84" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q84" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R84" s="2"/>
       <c r="S84" s="2" t="s">
@@ -6929,10 +6953,10 @@
         <v>231</v>
       </c>
       <c r="V84" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="85" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -6940,13 +6964,13 @@
         <v>22</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>50</v>
@@ -6962,19 +6986,19 @@
         <v>326</v>
       </c>
       <c r="M85" s="2" t="s">
-        <v>452</v>
+        <v>578</v>
       </c>
       <c r="N85" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O85" s="2" t="s">
-        <v>453</v>
+        <v>446</v>
       </c>
       <c r="P85" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q85" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q85" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R85" s="2"/>
       <c r="S85" s="2" t="s">
@@ -6987,10 +7011,10 @@
         <v>231</v>
       </c>
       <c r="V85" s="2" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="86" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -6998,13 +7022,13 @@
         <v>22</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>50</v>
@@ -7040,7 +7064,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="87" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -7048,13 +7072,13 @@
         <v>22</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>50</v>
@@ -7090,7 +7114,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="88" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -7098,13 +7122,13 @@
         <v>22</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>50</v>
@@ -7140,7 +7164,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="89" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -7148,13 +7172,13 @@
         <v>22</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>50</v>
@@ -7170,19 +7194,19 @@
         <v>326</v>
       </c>
       <c r="M89" s="2" t="s">
-        <v>467</v>
+        <v>580</v>
       </c>
       <c r="N89" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O89" s="2" t="s">
-        <v>468</v>
+        <v>459</v>
       </c>
       <c r="P89" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q89" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q89" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R89" s="2"/>
       <c r="S89" s="2" t="s">
@@ -7195,10 +7219,10 @@
         <v>231</v>
       </c>
       <c r="V89" s="2" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="90" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -7206,13 +7230,13 @@
         <v>22</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>471</v>
+        <v>461</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>472</v>
+        <v>462</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>50</v>
@@ -7228,19 +7252,19 @@
         <v>326</v>
       </c>
       <c r="M90" s="2" t="s">
-        <v>473</v>
+        <v>582</v>
       </c>
       <c r="N90" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O90" s="2" t="s">
-        <v>474</v>
+        <v>463</v>
       </c>
       <c r="P90" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q90" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q90" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R90" s="2"/>
       <c r="S90" s="2" t="s">
@@ -7253,10 +7277,10 @@
         <v>231</v>
       </c>
       <c r="V90" s="2" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="91" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -7264,13 +7288,13 @@
         <v>22</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>476</v>
+        <v>464</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>477</v>
+        <v>465</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>478</v>
+        <v>466</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>50</v>
@@ -7286,19 +7310,19 @@
         <v>326</v>
       </c>
       <c r="M91" s="2" t="s">
-        <v>479</v>
+        <v>584</v>
       </c>
       <c r="N91" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O91" s="2" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="P91" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q91" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q91" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R91" s="2"/>
       <c r="S91" s="2" t="s">
@@ -7311,10 +7335,10 @@
         <v>231</v>
       </c>
       <c r="V91" s="2" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="92" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -7322,13 +7346,13 @@
         <v>22</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>482</v>
+        <v>468</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>484</v>
+        <v>470</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>50</v>
@@ -7344,19 +7368,19 @@
         <v>326</v>
       </c>
       <c r="M92" s="2" t="s">
-        <v>485</v>
+        <v>586</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O92" s="2" t="s">
-        <v>486</v>
+        <v>471</v>
       </c>
       <c r="P92" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q92" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q92" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R92" s="2"/>
       <c r="S92" s="2" t="s">
@@ -7369,10 +7393,10 @@
         <v>231</v>
       </c>
       <c r="V92" s="2" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="93" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -7380,13 +7404,13 @@
         <v>22</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>488</v>
+        <v>472</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>489</v>
+        <v>473</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>490</v>
+        <v>474</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>50</v>
@@ -7422,7 +7446,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -7430,13 +7454,13 @@
         <v>22</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>491</v>
+        <v>475</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>492</v>
+        <v>476</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>493</v>
+        <v>477</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>50</v>
@@ -7452,19 +7476,19 @@
         <v>326</v>
       </c>
       <c r="M94" s="2" t="s">
-        <v>494</v>
+        <v>588</v>
       </c>
       <c r="N94" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O94" s="2" t="s">
-        <v>495</v>
+        <v>478</v>
       </c>
       <c r="P94" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q94" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q94" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R94" s="2"/>
       <c r="S94" s="2" t="s">
@@ -7477,10 +7501,10 @@
         <v>231</v>
       </c>
       <c r="V94" s="2" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="95" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -7488,13 +7512,13 @@
         <v>22</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>497</v>
+        <v>479</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>498</v>
+        <v>480</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>499</v>
+        <v>481</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>50</v>
@@ -7530,7 +7554,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="96" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -7538,13 +7562,13 @@
         <v>22</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>500</v>
+        <v>482</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>501</v>
+        <v>483</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>502</v>
+        <v>484</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>50</v>
@@ -7580,7 +7604,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="97" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -7588,13 +7612,13 @@
         <v>22</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>503</v>
+        <v>485</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>504</v>
+        <v>486</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>505</v>
+        <v>487</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>50</v>
@@ -7630,7 +7654,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -7638,13 +7662,13 @@
         <v>22</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>507</v>
+        <v>489</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>508</v>
+        <v>490</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>50</v>
@@ -7680,7 +7704,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="99" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -7688,13 +7712,13 @@
         <v>22</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>509</v>
+        <v>491</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>510</v>
+        <v>492</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>50</v>
@@ -7710,19 +7734,19 @@
         <v>326</v>
       </c>
       <c r="M99" s="2" t="s">
-        <v>512</v>
+        <v>590</v>
       </c>
       <c r="N99" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O99" s="2" t="s">
-        <v>513</v>
+        <v>494</v>
       </c>
       <c r="P99" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q99" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q99" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R99" s="2"/>
       <c r="S99" s="2" t="s">
@@ -7735,10 +7759,10 @@
         <v>231</v>
       </c>
       <c r="V99" s="2" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="100" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="100" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -7746,13 +7770,13 @@
         <v>22</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>515</v>
+        <v>495</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>516</v>
+        <v>496</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>517</v>
+        <v>497</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>50</v>
@@ -7768,19 +7792,19 @@
         <v>326</v>
       </c>
       <c r="M100" s="2" t="s">
-        <v>518</v>
+        <v>592</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O100" s="2" t="s">
-        <v>519</v>
+        <v>498</v>
       </c>
       <c r="P100" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q100" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="Q100" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="R100" s="2"/>
       <c r="S100" s="2" t="s">
@@ -7793,10 +7817,10 @@
         <v>231</v>
       </c>
       <c r="V100" s="2" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="101" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="101" spans="1:22" ht="280" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -7804,13 +7828,13 @@
         <v>22</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>521</v>
+        <v>499</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>522</v>
+        <v>500</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>523</v>
+        <v>501</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>50</v>
@@ -7819,20 +7843,20 @@
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2" t="s">
-        <v>524</v>
+        <v>502</v>
       </c>
       <c r="K101" s="2"/>
       <c r="L101" s="2" t="s">
         <v>326</v>
       </c>
       <c r="M101" s="2" t="s">
-        <v>525</v>
+        <v>503</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>526</v>
+        <v>504</v>
       </c>
       <c r="O101" s="2" t="s">
-        <v>527</v>
+        <v>505</v>
       </c>
       <c r="P101" s="2" t="s">
         <v>346</v>
@@ -7854,7 +7878,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -7862,13 +7886,13 @@
         <v>22</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>528</v>
+        <v>506</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>529</v>
+        <v>507</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>530</v>
+        <v>508</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>50</v>
@@ -7877,20 +7901,20 @@
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2" t="s">
-        <v>531</v>
+        <v>509</v>
       </c>
       <c r="K102" s="2"/>
       <c r="L102" s="2" t="s">
         <v>326</v>
       </c>
       <c r="M102" s="2" t="s">
-        <v>532</v>
+        <v>510</v>
       </c>
       <c r="N102" s="2" t="s">
-        <v>529</v>
+        <v>507</v>
       </c>
       <c r="O102" s="2" t="s">
-        <v>533</v>
+        <v>511</v>
       </c>
       <c r="P102" s="2" t="s">
         <v>346</v>
@@ -7912,7 +7936,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -7920,13 +7944,13 @@
         <v>22</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>534</v>
+        <v>512</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>535</v>
+        <v>513</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>536</v>
+        <v>514</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>50</v>
@@ -7935,20 +7959,20 @@
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
       <c r="J103" s="2" t="s">
-        <v>531</v>
+        <v>509</v>
       </c>
       <c r="K103" s="2"/>
       <c r="L103" s="2" t="s">
         <v>326</v>
       </c>
       <c r="M103" s="2" t="s">
-        <v>537</v>
+        <v>515</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>538</v>
+        <v>516</v>
       </c>
       <c r="O103" s="2" t="s">
-        <v>539</v>
+        <v>517</v>
       </c>
       <c r="P103" s="2" t="s">
         <v>346</v>
@@ -7970,7 +7994,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -7978,13 +8002,13 @@
         <v>22</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>540</v>
+        <v>518</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>541</v>
+        <v>519</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>541</v>
+        <v>519</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>50</v>
@@ -7993,20 +8017,20 @@
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2" t="s">
-        <v>542</v>
+        <v>520</v>
       </c>
       <c r="K104" s="2"/>
       <c r="L104" s="2" t="s">
         <v>326</v>
       </c>
       <c r="M104" s="3" t="s">
-        <v>585</v>
+        <v>563</v>
       </c>
       <c r="N104" s="3" t="s">
-        <v>586</v>
+        <v>564</v>
       </c>
       <c r="O104" s="3" t="s">
-        <v>587</v>
+        <v>565</v>
       </c>
       <c r="P104" s="3" t="s">
         <v>400</v>
@@ -8025,10 +8049,10 @@
         <v>231</v>
       </c>
       <c r="V104" s="3" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="105" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -8036,13 +8060,13 @@
         <v>22</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>543</v>
+        <v>521</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>544</v>
+        <v>522</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>544</v>
+        <v>522</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>50</v>
@@ -8051,26 +8075,26 @@
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
       <c r="J105" s="2" t="s">
-        <v>545</v>
+        <v>523</v>
       </c>
       <c r="K105" s="2"/>
       <c r="L105" s="2" t="s">
         <v>326</v>
       </c>
       <c r="M105" s="3" t="s">
-        <v>591</v>
+        <v>569</v>
       </c>
       <c r="N105" s="3" t="s">
-        <v>590</v>
+        <v>568</v>
       </c>
       <c r="O105" s="3" t="s">
-        <v>589</v>
+        <v>567</v>
       </c>
       <c r="P105" s="3" t="s">
         <v>346</v>
       </c>
       <c r="Q105" s="3" t="s">
-        <v>588</v>
+        <v>566</v>
       </c>
       <c r="R105" s="2"/>
       <c r="S105" s="2" t="s">
@@ -8086,7 +8110,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:22" ht="266" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -8094,13 +8118,13 @@
         <v>22</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>546</v>
+        <v>524</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>547</v>
+        <v>525</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>547</v>
+        <v>525</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>50</v>
@@ -8109,20 +8133,20 @@
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2" t="s">
-        <v>545</v>
+        <v>523</v>
       </c>
       <c r="K106" s="2"/>
       <c r="L106" s="3" t="s">
         <v>326</v>
       </c>
       <c r="M106" s="3" t="s">
-        <v>592</v>
+        <v>570</v>
       </c>
       <c r="N106" s="3" t="s">
-        <v>590</v>
+        <v>568</v>
       </c>
       <c r="O106" s="3" t="s">
-        <v>589</v>
+        <v>567</v>
       </c>
       <c r="P106" s="3" t="s">
         <v>346</v>
@@ -8144,7 +8168,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -8152,13 +8176,13 @@
         <v>22</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>548</v>
+        <v>526</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>549</v>
+        <v>527</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>549</v>
+        <v>527</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>50</v>
@@ -8167,7 +8191,7 @@
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2" t="s">
-        <v>550</v>
+        <v>528</v>
       </c>
       <c r="K107" s="2"/>
       <c r="L107" s="2"/>
@@ -8192,7 +8216,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="108" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -8200,13 +8224,13 @@
         <v>22</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>551</v>
+        <v>529</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>552</v>
+        <v>530</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>552</v>
+        <v>530</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>50</v>
@@ -8215,7 +8239,7 @@
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2" t="s">
-        <v>553</v>
+        <v>531</v>
       </c>
       <c r="K108" s="2"/>
       <c r="L108" s="2"/>
@@ -8240,7 +8264,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="109" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -8248,13 +8272,13 @@
         <v>22</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>554</v>
+        <v>532</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>555</v>
+        <v>533</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>555</v>
+        <v>533</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>50</v>
@@ -8263,7 +8287,7 @@
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
       <c r="J109" s="2" t="s">
-        <v>556</v>
+        <v>534</v>
       </c>
       <c r="K109" s="2"/>
       <c r="L109" s="2"/>
@@ -8288,7 +8312,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="110" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -8296,13 +8320,13 @@
         <v>22</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>557</v>
+        <v>535</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>558</v>
+        <v>536</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>558</v>
+        <v>536</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>50</v>
@@ -8311,7 +8335,7 @@
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
       <c r="J110" s="2" t="s">
-        <v>559</v>
+        <v>537</v>
       </c>
       <c r="K110" s="2"/>
       <c r="L110" s="2"/>
@@ -8336,7 +8360,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="111" spans="1:22" ht="99.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:22" ht="98" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -8344,13 +8368,13 @@
         <v>22</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>560</v>
+        <v>538</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>561</v>
+        <v>539</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>561</v>
+        <v>539</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>50</v>
@@ -8359,10 +8383,10 @@
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
       <c r="J111" s="2" t="s">
-        <v>562</v>
+        <v>540</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>563</v>
+        <v>541</v>
       </c>
       <c r="L111" s="2"/>
       <c r="M111" s="2" t="s">
@@ -8386,7 +8410,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="112" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -8394,13 +8418,13 @@
         <v>22</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>564</v>
+        <v>542</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>565</v>
+        <v>543</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>565</v>
+        <v>543</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>50</v>
@@ -8409,7 +8433,7 @@
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2" t="s">
-        <v>553</v>
+        <v>531</v>
       </c>
       <c r="K112" s="2"/>
       <c r="L112" s="2"/>
@@ -8434,7 +8458,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="113" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:22" ht="42" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -8442,13 +8466,13 @@
         <v>22</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>566</v>
+        <v>544</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>567</v>
+        <v>545</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>567</v>
+        <v>545</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>50</v>
@@ -8457,7 +8481,7 @@
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2" t="s">
-        <v>553</v>
+        <v>531</v>
       </c>
       <c r="K113" s="2"/>
       <c r="L113" s="2"/>
@@ -8482,7 +8506,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="114" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:22" ht="28" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -8490,13 +8514,13 @@
         <v>22</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>568</v>
+        <v>546</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>569</v>
+        <v>547</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>570</v>
+        <v>548</v>
       </c>
       <c r="F114" s="2" t="s">
         <v>50</v>
@@ -8518,19 +8542,19 @@
       <c r="Q114" s="2"/>
       <c r="R114" s="2"/>
       <c r="S114" s="2" t="s">
-        <v>593</v>
+        <v>571</v>
       </c>
       <c r="T114" s="2" t="s">
-        <v>593</v>
+        <v>571</v>
       </c>
       <c r="U114" s="2" t="s">
-        <v>593</v>
+        <v>571</v>
       </c>
       <c r="V114" s="2" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -8538,13 +8562,13 @@
         <v>22</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>571</v>
+        <v>549</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>572</v>
+        <v>550</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>572</v>
+        <v>550</v>
       </c>
       <c r="F115" s="2" t="s">
         <v>50</v>
@@ -8576,7 +8600,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -8584,13 +8608,13 @@
         <v>22</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>573</v>
+        <v>551</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>574</v>
+        <v>552</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>574</v>
+        <v>552</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>50</v>
@@ -8622,7 +8646,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -8630,13 +8654,13 @@
         <v>22</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>575</v>
+        <v>553</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>576</v>
+        <v>554</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>576</v>
+        <v>554</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>50</v>

</xml_diff>

<commit_message>
set med lipid lowering undetermined for now
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NES.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A81ADA-E275-4395-9B64-2079F5F53381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4890413-676E-4EF2-8B5F-86FAB1FA6C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_processing_elements" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1559" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="602">
   <si>
     <t>index</t>
   </si>
@@ -1921,11 +1921,6 @@
 Dyslipidemia_medication == 1 | Dyslipidemia_statins == 1 | Dyslipidemia_medication_cholesterol_lowering == 1 ~ 1L;
 Dyslipidemia_medication == 0 ~ 0L;
 ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>Dyslipidemia_medication;
-Dyslipidemia_statins;
-Dyslipidemia_medication_cholesterol_lowering</t>
   </si>
   <si>
     <t>Use medication;
@@ -2260,7 +2255,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2566,7 +2561,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W117"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -2584,13 +2579,13 @@
     <col min="16" max="16" width="24" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="46" customWidth="1"/>
-    <col min="19" max="19" width="14.1796875" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="16" customWidth="1"/>
     <col min="22" max="22" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2658,10 +2653,10 @@
         <v>21</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2717,7 +2712,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2765,7 +2760,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="210" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" ht="213.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2813,7 +2808,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2861,7 +2856,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="42" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2893,7 +2888,7 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>59</v>
@@ -2918,10 +2913,10 @@
         <v>62</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2977,7 +2972,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="56" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" ht="57" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -3009,7 +3004,7 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>76</v>
@@ -3034,10 +3029,10 @@
         <v>62</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="126" x14ac:dyDescent="0.35">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3089,7 +3084,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="56" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" ht="57" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3141,7 +3136,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="140" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3191,7 +3186,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="42" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3243,7 +3238,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3291,7 +3286,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3337,7 +3332,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="112" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" ht="114" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3387,7 +3382,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="70" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3435,7 +3430,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3487,7 +3482,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3539,7 +3534,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3587,7 +3582,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3639,7 +3634,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3687,7 +3682,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3739,7 +3734,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3791,7 +3786,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3839,7 +3834,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3887,7 +3882,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3933,7 +3928,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3985,7 +3980,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -4037,7 +4032,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -4089,7 +4084,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -4141,7 +4136,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -4189,7 +4184,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -4237,7 +4232,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -4285,7 +4280,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -4333,7 +4328,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -4381,7 +4376,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -4429,7 +4424,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="98" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:23" ht="114" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -4479,7 +4474,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -4527,7 +4522,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -4575,7 +4570,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="70" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4627,7 +4622,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="56" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:23" ht="57" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4677,7 +4672,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="70" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4729,7 +4724,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="42" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4781,7 +4776,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -4829,7 +4824,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="336" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:23" ht="342" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -4877,22 +4872,22 @@
       </c>
       <c r="R45" s="2"/>
       <c r="S45" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="T45" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="U45" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="V45" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="W45" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="70" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -4950,7 +4945,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="84" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:23" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -5012,7 +5007,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="28" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -5062,7 +5057,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -5114,7 +5109,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -5162,7 +5157,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="154" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -5212,7 +5207,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -5262,7 +5257,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -5312,7 +5307,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -5360,7 +5355,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -5408,7 +5403,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="154" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -5456,7 +5451,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -5506,7 +5501,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="58" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -5556,7 +5551,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -5606,7 +5601,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="84" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -5654,7 +5649,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -5704,7 +5699,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:22" ht="84" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -5754,7 +5749,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="112" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -5806,7 +5801,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -5856,7 +5851,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="65" spans="1:22" ht="70" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -5908,7 +5903,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="66" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -5956,7 +5951,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -6004,7 +5999,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="68" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -6054,7 +6049,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="69" spans="1:22" ht="392" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -6114,7 +6109,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="70" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -6176,7 +6171,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="71" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -6236,7 +6231,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="72" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -6296,7 +6291,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="73" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -6358,7 +6353,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="74" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -6418,7 +6413,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="75" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -6478,7 +6473,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="76" spans="1:22" ht="350" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" ht="370.5" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -6540,7 +6535,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="77" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -6600,7 +6595,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="78" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -6660,7 +6655,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="79" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -6722,7 +6717,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="80" spans="1:22" ht="56" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" ht="57" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -6782,7 +6777,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="81" spans="1:22" ht="196" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" ht="213.75" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -6842,7 +6837,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="82" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -6872,7 +6867,7 @@
         <v>322</v>
       </c>
       <c r="M82" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="N82" s="2" t="s">
         <v>427</v>
@@ -6897,10 +6892,10 @@
         <v>227</v>
       </c>
       <c r="V82" s="2" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="83" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -6930,7 +6925,7 @@
         <v>322</v>
       </c>
       <c r="M83" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="N83" s="2" t="s">
         <v>427</v>
@@ -6955,10 +6950,10 @@
         <v>227</v>
       </c>
       <c r="V83" s="2" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="84" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -6988,7 +6983,7 @@
         <v>322</v>
       </c>
       <c r="M84" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="N84" s="2" t="s">
         <v>427</v>
@@ -7013,10 +7008,10 @@
         <v>227</v>
       </c>
       <c r="V84" s="2" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="85" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -7046,7 +7041,7 @@
         <v>322</v>
       </c>
       <c r="M85" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N85" s="2" t="s">
         <v>427</v>
@@ -7071,10 +7066,10 @@
         <v>227</v>
       </c>
       <c r="V85" s="2" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="86" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -7104,7 +7099,7 @@
         <v>322</v>
       </c>
       <c r="M86" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -7121,10 +7116,10 @@
         <v>227</v>
       </c>
       <c r="V86" s="2" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="87" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -7154,7 +7149,7 @@
         <v>322</v>
       </c>
       <c r="M87" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -7171,10 +7166,10 @@
         <v>227</v>
       </c>
       <c r="V87" s="2" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="88" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -7204,7 +7199,7 @@
         <v>322</v>
       </c>
       <c r="M88" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -7221,10 +7216,10 @@
         <v>227</v>
       </c>
       <c r="V88" s="2" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="89" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -7254,7 +7249,7 @@
         <v>322</v>
       </c>
       <c r="M89" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="N89" s="2" t="s">
         <v>427</v>
@@ -7279,10 +7274,10 @@
         <v>227</v>
       </c>
       <c r="V89" s="2" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="90" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -7312,7 +7307,7 @@
         <v>322</v>
       </c>
       <c r="M90" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="N90" s="2" t="s">
         <v>427</v>
@@ -7337,10 +7332,10 @@
         <v>227</v>
       </c>
       <c r="V90" s="2" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="91" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -7370,7 +7365,7 @@
         <v>322</v>
       </c>
       <c r="M91" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="N91" s="2" t="s">
         <v>427</v>
@@ -7395,10 +7390,10 @@
         <v>227</v>
       </c>
       <c r="V91" s="2" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="92" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -7428,7 +7423,7 @@
         <v>322</v>
       </c>
       <c r="M92" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="N92" s="2" t="s">
         <v>427</v>
@@ -7453,10 +7448,10 @@
         <v>227</v>
       </c>
       <c r="V92" s="2" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="93" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -7506,7 +7501,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="94" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -7536,7 +7531,7 @@
         <v>322</v>
       </c>
       <c r="M94" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="N94" s="2" t="s">
         <v>427</v>
@@ -7561,10 +7556,10 @@
         <v>227</v>
       </c>
       <c r="V94" s="2" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="95" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -7594,7 +7589,7 @@
         <v>322</v>
       </c>
       <c r="M95" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -7611,10 +7606,10 @@
         <v>227</v>
       </c>
       <c r="V95" s="2" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="96" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -7664,7 +7659,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="97" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:23" ht="285" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -7714,7 +7709,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:23" ht="285" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -7764,7 +7759,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="99" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:23" ht="285" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -7794,7 +7789,7 @@
         <v>322</v>
       </c>
       <c r="M99" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="N99" s="2" t="s">
         <v>427</v>
@@ -7819,10 +7814,10 @@
         <v>227</v>
       </c>
       <c r="V99" s="2" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="100" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" ht="285" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -7852,7 +7847,7 @@
         <v>322</v>
       </c>
       <c r="M100" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="N100" s="2" t="s">
         <v>427</v>
@@ -7877,10 +7872,10 @@
         <v>227</v>
       </c>
       <c r="V100" s="2" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="101" spans="1:22" ht="280" x14ac:dyDescent="0.35">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -7938,7 +7933,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="102" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:23" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -7996,7 +7991,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="103" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:23" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -8054,7 +8049,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="104" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:23" ht="370.5" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -8083,14 +8078,14 @@
       <c r="L104" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="M104" s="3" t="s">
+      <c r="M104" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N104" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="N104" s="3" t="s">
+      <c r="O104" s="3" t="s">
         <v>560</v>
-      </c>
-      <c r="O104" s="3" t="s">
-        <v>561</v>
       </c>
       <c r="P104" s="3" t="s">
         <v>396</v>
@@ -8100,19 +8095,22 @@
       </c>
       <c r="R104" s="2"/>
       <c r="S104" s="2" t="s">
-        <v>32</v>
+        <v>566</v>
       </c>
       <c r="T104" s="2" t="s">
-        <v>40</v>
+        <v>566</v>
       </c>
       <c r="U104" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="V104" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="V104" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="W104" s="3" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="105" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:23" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -8142,19 +8140,19 @@
         <v>322</v>
       </c>
       <c r="M105" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="N105" s="3" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="O105" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="P105" s="3" t="s">
         <v>342</v>
       </c>
       <c r="Q105" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="R105" s="2"/>
       <c r="S105" s="2" t="s">
@@ -8170,7 +8168,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="106" spans="1:22" ht="266" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:23" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -8200,13 +8198,13 @@
         <v>322</v>
       </c>
       <c r="M106" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="N106" s="3" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="O106" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="P106" s="3" t="s">
         <v>342</v>
@@ -8228,7 +8226,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="107" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -8276,7 +8274,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="108" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -8324,7 +8322,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="109" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -8372,7 +8370,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="110" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -8420,7 +8418,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="111" spans="1:22" ht="98" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:23" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -8470,7 +8468,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="112" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -8518,7 +8516,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="113" spans="1:22" ht="42" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -8566,7 +8564,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="114" spans="1:22" ht="28" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -8602,19 +8600,19 @@
       <c r="Q114" s="2"/>
       <c r="R114" s="2"/>
       <c r="S114" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="T114" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="U114" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="V114" s="2" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.35">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -8660,7 +8658,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -8706,7 +8704,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>116</v>
       </c>

</xml_diff>

<commit_message>
Update DPE to remove mortality
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NES.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NES.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\NES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DF560B4-85F4-46B3-8E3A-E6C20BC6C2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8139E28B-4502-46C1-B270-790961039887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_processing_elements" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_processing_elements!$A$1:$V$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_processing_elements!$A$1:$V$113</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="594">
   <si>
     <t>index</t>
   </si>
@@ -733,9 +733,6 @@
     <t>Record study-specific data-collection methods and question wording, including the types of alcohol included.</t>
   </si>
   <si>
-    <t>Alcohol_change_glasses</t>
-  </si>
-  <si>
     <t>Current alcohol consumption (glasses/week)</t>
   </si>
   <si>
@@ -743,12 +740,6 @@
   </si>
   <si>
     <t>case_when</t>
-  </si>
-  <si>
-    <t>case_when(
-is.na(Alcohol_change_glasses) | Alcohol_change_glasses == "." ~ NA_real_;
-Alcohol_change_glasses &gt;= 0 ~ as.numeric(Alcohol_change_glasses)*10;
-ELSE ~ NA_real_)</t>
   </si>
   <si>
     <t>lsb_alc_freq</t>
@@ -778,9 +769,6 @@
     <t>0 = Never smoked ; 
 1 = Previously smoked ; 
 2 = Currently smoke</t>
-  </si>
-  <si>
-    <t>Smoker_change</t>
   </si>
   <si>
     <t>Change in smoking behavior</t>
@@ -1864,33 +1852,6 @@
     <t>Montreal Cognitive Assessment (MoCA) score</t>
   </si>
   <si>
-    <t>dth_status</t>
-  </si>
-  <si>
-    <t>Death status</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is deceased</t>
-  </si>
-  <si>
-    <t>dth_date_day</t>
-  </si>
-  <si>
-    <t>Death date - Day</t>
-  </si>
-  <si>
-    <t>dth_date_month</t>
-  </si>
-  <si>
-    <t>Death date - Month</t>
-  </si>
-  <si>
-    <t>dth_date_year</t>
-  </si>
-  <si>
-    <t>Death date - Year</t>
-  </si>
-  <si>
     <t>Consumption frequency was not collected; only quantity (glasses per week) is available. Frequency could in principle be banded from quantity, but the "Monthly" category is unreachable from a weekly count</t>
   </si>
   <si>
@@ -2182,6 +2143,19 @@
   </si>
   <si>
     <t>lubridate::interval(as.Date(date_birth),as.Date(last_fu)) %/% lubridate::years(1)</t>
+  </si>
+  <si>
+    <t>case_when(
+is.na(Alcohol_change_glasses) | Alcohol_change_glasses == "." ~ NA_real_;
+Alcohol_change_glasses &gt;= 0 ~ as.numeric(Alcohol_change_glasses)*10;
+ELSE ~ NA_real_)
+2026-08-31: Created a version without input variables: Alcohol_change_glasses.</t>
+  </si>
+  <si>
+    <t>2026-08-31: Created a version without input variables: Alcohol_change_glasses.</t>
+  </si>
+  <si>
+    <t>2026-08-31: Created a version without input variables: Smoker_change.</t>
   </si>
 </sst>
 </file>
@@ -2209,6 +2183,7 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2255,13 +2230,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2566,33 +2539,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W117"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:W113"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="36" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="11" width="34" customWidth="1"/>
-    <col min="12" max="12" width="38" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
-    <col min="14" max="14" width="26" customWidth="1"/>
-    <col min="15" max="15" width="40" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="17" width="12" customWidth="1"/>
-    <col min="18" max="18" width="46" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" customWidth="1"/>
-    <col min="20" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
-    <col min="22" max="22" width="52" customWidth="1"/>
-    <col min="23" max="23" width="37.42578125" customWidth="1"/>
+    <col min="1" max="1" width="6" style="4" customWidth="1"/>
+    <col min="2" max="2" width="11" style="4" customWidth="1"/>
+    <col min="3" max="4" width="30" style="4" customWidth="1"/>
+    <col min="5" max="5" width="36" style="4" customWidth="1"/>
+    <col min="6" max="6" width="9" style="4" customWidth="1"/>
+    <col min="7" max="7" width="10" style="4" customWidth="1"/>
+    <col min="8" max="8" width="11" style="4" customWidth="1"/>
+    <col min="9" max="9" width="24" style="4" customWidth="1"/>
+    <col min="10" max="11" width="34" style="4" customWidth="1"/>
+    <col min="12" max="12" width="38" style="4" customWidth="1"/>
+    <col min="13" max="13" width="24" style="4" customWidth="1"/>
+    <col min="14" max="14" width="26" style="4" customWidth="1"/>
+    <col min="15" max="15" width="40" style="4" customWidth="1"/>
+    <col min="16" max="16" width="24" style="4" customWidth="1"/>
+    <col min="17" max="17" width="12" style="4" customWidth="1"/>
+    <col min="18" max="18" width="46" style="4" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" style="4" customWidth="1"/>
+    <col min="20" max="20" width="15" style="4" customWidth="1"/>
+    <col min="21" max="21" width="16" style="4" customWidth="1"/>
+    <col min="22" max="22" width="52" style="4" customWidth="1"/>
+    <col min="23" max="23" width="37.42578125" style="4" customWidth="1"/>
+    <col min="24" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2659,11 +2633,11 @@
       <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="4" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="W1" s="3" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2719,7 +2693,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2767,7 +2741,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="213.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="213.75" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2815,7 +2789,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2863,7 +2837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2895,7 +2869,7 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>597</v>
+        <v>585</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>59</v>
@@ -2920,10 +2894,10 @@
         <v>62</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2979,7 +2953,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="57" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="57" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -3011,7 +2985,7 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>599</v>
+        <v>587</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>76</v>
@@ -3036,13 +3010,13 @@
         <v>62</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>602</v>
+        <v>590</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="128.25" x14ac:dyDescent="0.25">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3094,7 +3068,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="57" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="57" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3146,7 +3120,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="142.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3196,7 +3170,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3248,7 +3222,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3296,7 +3270,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3342,7 +3316,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="114" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="114" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3392,7 +3366,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3440,7 +3414,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3492,7 +3466,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3544,7 +3518,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3592,7 +3566,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3644,7 +3618,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3692,7 +3666,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3744,7 +3718,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3796,7 +3770,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3844,7 +3818,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3892,7 +3866,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3938,7 +3912,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" ht="57" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3990,7 +3964,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" ht="57" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -4042,7 +4016,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" ht="57" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -4094,7 +4068,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -4146,7 +4120,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -4194,7 +4168,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -4242,7 +4216,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -4290,7 +4264,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -4338,7 +4312,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -4386,7 +4360,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -4434,7 +4408,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="114" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:23" ht="114" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -4484,7 +4458,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -4532,7 +4506,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -4580,7 +4554,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4632,7 +4606,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="57" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4682,7 +4656,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4734,7 +4708,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4786,7 +4760,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -4834,7 +4808,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="342" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -4866,13 +4840,13 @@
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N45" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="N45" s="2" t="s">
+      <c r="O45" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="O45" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="P45" s="2" t="s">
         <v>31</v>
@@ -4882,22 +4856,22 @@
       </c>
       <c r="R45" s="2"/>
       <c r="S45" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="T45" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="U45" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="V45" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="W45" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="46" spans="1:23" ht="71.25" x14ac:dyDescent="0.25">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -4905,13 +4879,13 @@
         <v>22</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>50</v>
@@ -4922,16 +4896,16 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="M46" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N46" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="N46" s="2" t="s">
+      <c r="O46" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="O46" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="P46" s="2" t="s">
         <v>31</v>
@@ -4940,7 +4914,7 @@
         <v>31</v>
       </c>
       <c r="R46" s="2" t="s">
-        <v>551</v>
+        <v>539</v>
       </c>
       <c r="S46" s="2" t="s">
         <v>86</v>
@@ -4954,8 +4928,11 @@
       <c r="V46" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="47" spans="1:23" ht="99.75" x14ac:dyDescent="0.25">
+      <c r="W46" s="2" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -4963,13 +4940,13 @@
         <v>22</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>50</v>
@@ -4978,37 +4955,37 @@
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="L47" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="M47" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N47" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="L47" s="2" t="s">
+      <c r="O47" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="P47" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="N47" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="O47" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="P47" s="2" t="s">
-        <v>240</v>
       </c>
       <c r="Q47" s="2" t="s">
         <v>31</v>
       </c>
       <c r="R47" s="2" t="s">
-        <v>552</v>
+        <v>540</v>
       </c>
       <c r="S47" s="2" t="s">
         <v>86</v>
       </c>
       <c r="T47" s="2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="U47" s="2" t="s">
         <v>86</v>
@@ -5016,8 +4993,11 @@
       <c r="V47" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="48" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="W47" s="4" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -5025,13 +5005,13 @@
         <v>22</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>50</v>
@@ -5041,10 +5021,10 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="M48" s="2" t="s">
         <v>39</v>
@@ -5067,7 +5047,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -5075,27 +5055,27 @@
         <v>22</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>105</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="2" t="s">
@@ -5119,7 +5099,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -5127,13 +5107,13 @@
         <v>22</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>105</v>
@@ -5167,7 +5147,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="171" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:22" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -5175,13 +5155,13 @@
         <v>22</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>50</v>
@@ -5190,11 +5170,11 @@
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="K51" s="2"/>
       <c r="L51" s="2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="M51" s="2" t="s">
         <v>39</v>
@@ -5217,7 +5197,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:22" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -5225,13 +5205,13 @@
         <v>22</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>50</v>
@@ -5241,10 +5221,10 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>39</v>
@@ -5267,7 +5247,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -5275,13 +5255,13 @@
         <v>22</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>50</v>
@@ -5290,11 +5270,11 @@
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="K53" s="2"/>
       <c r="L53" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>39</v>
@@ -5317,7 +5297,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -5325,13 +5305,13 @@
         <v>22</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>50</v>
@@ -5342,7 +5322,7 @@
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M54" s="2" t="s">
         <v>39</v>
@@ -5365,7 +5345,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -5373,13 +5353,13 @@
         <v>22</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>50</v>
@@ -5390,7 +5370,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M55" s="2" t="s">
         <v>39</v>
@@ -5413,7 +5393,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="156.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:22" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -5421,13 +5401,13 @@
         <v>22</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>50</v>
@@ -5438,7 +5418,7 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="M56" s="2" t="s">
         <v>39</v>
@@ -5461,7 +5441,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -5469,13 +5449,13 @@
         <v>22</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>50</v>
@@ -5484,11 +5464,11 @@
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="K57" s="2"/>
       <c r="L57" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M57" s="2" t="s">
         <v>39</v>
@@ -5511,7 +5491,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="58" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -5519,13 +5499,13 @@
         <v>22</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>50</v>
@@ -5534,11 +5514,11 @@
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="K58" s="2"/>
       <c r="L58" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M58" s="2" t="s">
         <v>39</v>
@@ -5561,7 +5541,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -5569,13 +5549,13 @@
         <v>22</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>105</v>
@@ -5586,7 +5566,7 @@
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>
@@ -5611,7 +5591,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:22" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -5619,13 +5599,13 @@
         <v>22</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>50</v>
@@ -5636,7 +5616,7 @@
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
       <c r="L60" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="M60" s="2" t="s">
         <v>39</v>
@@ -5659,7 +5639,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -5667,13 +5647,13 @@
         <v>22</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>50</v>
@@ -5683,10 +5663,10 @@
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="M61" s="2" t="s">
         <v>39</v>
@@ -5709,7 +5689,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:22" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:22" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -5717,13 +5697,13 @@
         <v>22</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>50</v>
@@ -5733,10 +5713,10 @@
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>39</v>
@@ -5759,7 +5739,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="128.25" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:22" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -5767,13 +5747,13 @@
         <v>22</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>50</v>
@@ -5782,10 +5762,10 @@
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L63" s="2" t="s">
         <v>91</v>
@@ -5811,7 +5791,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:22" ht="57" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -5819,13 +5799,13 @@
         <v>22</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>50</v>
@@ -5834,7 +5814,7 @@
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="K64" s="2"/>
       <c r="L64" s="2" t="s">
@@ -5861,7 +5841,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="65" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -5869,13 +5849,13 @@
         <v>22</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>50</v>
@@ -5884,10 +5864,10 @@
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>91</v>
@@ -5913,7 +5893,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="66" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -5921,13 +5901,13 @@
         <v>22</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>105</v>
@@ -5936,7 +5916,7 @@
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K66" s="2"/>
       <c r="L66" s="2"/>
@@ -5961,7 +5941,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -5969,19 +5949,19 @@
         <v>22</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>50</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
@@ -6009,7 +5989,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="68" spans="1:22" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:22" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -6017,13 +5997,13 @@
         <v>22</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>50</v>
@@ -6033,10 +6013,10 @@
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
       <c r="K68" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="M68" s="2" t="s">
         <v>39</v>
@@ -6059,7 +6039,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="69" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:22" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -6067,13 +6047,13 @@
         <v>22</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>50</v>
@@ -6082,28 +6062,28 @@
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M69" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="K69" s="2" t="s">
+      <c r="N69" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="L69" s="2" t="s">
+      <c r="O69" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="M69" s="2" t="s">
+      <c r="P69" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="N69" s="2" t="s">
+      <c r="Q69" s="2" t="s">
         <v>324</v>
-      </c>
-      <c r="O69" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="P69" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="Q69" s="2" t="s">
-        <v>327</v>
       </c>
       <c r="R69" s="2"/>
       <c r="S69" s="2" t="s">
@@ -6113,13 +6093,13 @@
         <v>40</v>
       </c>
       <c r="U69" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V69" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="70" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -6127,13 +6107,13 @@
         <v>22</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>50</v>
@@ -6141,32 +6121,32 @@
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="J70" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K70" s="2"/>
       <c r="L70" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="M70" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="O70" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="P70" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="N70" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="O70" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="P70" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="Q70" s="3" t="s">
+      <c r="Q70" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R70" s="3" t="s">
-        <v>553</v>
+      <c r="R70" s="2" t="s">
+        <v>541</v>
       </c>
       <c r="S70" s="2" t="s">
         <v>32</v>
@@ -6175,13 +6155,13 @@
         <v>40</v>
       </c>
       <c r="U70" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="V70" s="3" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="71" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="V70" s="2" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -6189,13 +6169,13 @@
         <v>22</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>50</v>
@@ -6203,26 +6183,26 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="J71" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K71" s="2"/>
       <c r="L71" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M71" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="N71" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="O71" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="P71" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="N71" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="O71" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="P71" s="2" t="s">
-        <v>342</v>
       </c>
       <c r="Q71" s="2" t="s">
         <v>31</v>
@@ -6238,10 +6218,10 @@
         <v>68</v>
       </c>
       <c r="V71" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="72" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -6249,13 +6229,13 @@
         <v>22</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>50</v>
@@ -6263,26 +6243,26 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K72" s="2"/>
       <c r="L72" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="O72" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="P72" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q72" s="2" t="s">
         <v>31</v>
@@ -6298,10 +6278,10 @@
         <v>68</v>
       </c>
       <c r="V72" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="73" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="73" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -6309,13 +6289,13 @@
         <v>22</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>50</v>
@@ -6323,32 +6303,32 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K73" s="2"/>
       <c r="L73" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M73" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="O73" s="3" t="s">
-        <v>357</v>
+        <v>353</v>
+      </c>
+      <c r="O73" s="2" t="s">
+        <v>354</v>
       </c>
       <c r="P73" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q73" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R73" s="3" t="s">
-        <v>555</v>
+      <c r="R73" s="2" t="s">
+        <v>543</v>
       </c>
       <c r="S73" s="2" t="s">
         <v>32</v>
@@ -6360,10 +6340,10 @@
         <v>68</v>
       </c>
       <c r="V73" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="74" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -6371,13 +6351,13 @@
         <v>22</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>50</v>
@@ -6385,26 +6365,26 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K74" s="2"/>
       <c r="L74" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M74" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="O74" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="P74" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q74" s="2" t="s">
         <v>31</v>
@@ -6420,10 +6400,10 @@
         <v>68</v>
       </c>
       <c r="V74" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="75" spans="1:22" ht="327.75" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -6431,13 +6411,13 @@
         <v>22</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>50</v>
@@ -6445,26 +6425,26 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="J75" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="K75" s="2"/>
       <c r="L75" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M75" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="O75" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="P75" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q75" s="2" t="s">
         <v>31</v>
@@ -6480,10 +6460,10 @@
         <v>68</v>
       </c>
       <c r="V75" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="76" spans="1:22" ht="399" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="76" spans="1:22" ht="399" x14ac:dyDescent="0.2">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -6491,13 +6471,13 @@
         <v>22</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>50</v>
@@ -6505,28 +6485,28 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="L76" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M76" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="J76" s="2" t="s">
+      <c r="N76" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="K76" s="2" t="s">
+      <c r="O76" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="L76" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="M76" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="N76" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="O76" s="2" t="s">
-        <v>380</v>
-      </c>
       <c r="P76" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q76" s="2" t="s">
         <v>31</v>
@@ -6542,10 +6522,10 @@
         <v>68</v>
       </c>
       <c r="V76" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="77" spans="1:22" ht="299.25" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -6553,13 +6533,13 @@
         <v>22</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>50</v>
@@ -6567,26 +6547,26 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="J77" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="K77" s="2"/>
       <c r="L77" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M77" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="N77" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="O77" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="P77" s="2" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="Q77" s="2" t="s">
         <v>78</v>
@@ -6599,13 +6579,13 @@
         <v>40</v>
       </c>
       <c r="U77" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="V77" s="3" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="78" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="V77" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -6613,13 +6593,13 @@
         <v>22</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>50</v>
@@ -6627,29 +6607,29 @@
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="J78" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="K78" s="2"/>
       <c r="L78" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M78" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="N78" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="O78" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="P78" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="N78" s="2" t="s">
+      <c r="Q78" s="2" t="s">
         <v>394</v>
-      </c>
-      <c r="O78" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="P78" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="Q78" s="2" t="s">
-        <v>397</v>
       </c>
       <c r="R78" s="2"/>
       <c r="S78" s="2" t="s">
@@ -6659,13 +6639,13 @@
         <v>40</v>
       </c>
       <c r="U78" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V78" s="2" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="79" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="79" spans="1:22" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -6673,13 +6653,13 @@
         <v>22</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>50</v>
@@ -6687,28 +6667,28 @@
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="L79" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M79" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="N79" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="J79" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="K79" s="2" t="s">
+      <c r="O79" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="L79" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="M79" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="N79" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="O79" s="2" t="s">
-        <v>406</v>
-      </c>
       <c r="P79" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q79" s="2" t="s">
         <v>31</v>
@@ -6724,10 +6704,10 @@
         <v>68</v>
       </c>
       <c r="V79" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="80" spans="1:22" ht="57" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" ht="57" x14ac:dyDescent="0.2">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -6735,13 +6715,13 @@
         <v>22</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>50</v>
@@ -6751,28 +6731,28 @@
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="L80" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="M80" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="N80" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="L80" s="2" t="s">
+      <c r="O80" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="M80" s="2" t="s">
+      <c r="P80" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="N80" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="O80" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="P80" s="2" t="s">
-        <v>414</v>
       </c>
       <c r="Q80" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R80" s="3" t="s">
-        <v>557</v>
+      <c r="R80" s="2" t="s">
+        <v>545</v>
       </c>
       <c r="S80" s="2" t="s">
         <v>32</v>
@@ -6787,7 +6767,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="81" spans="1:22" ht="228" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:22" ht="228" x14ac:dyDescent="0.2">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -6795,13 +6775,13 @@
         <v>22</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>50</v>
@@ -6810,25 +6790,25 @@
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="L81" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M81" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="N81" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="K81" s="2" t="s">
+      <c r="O81" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="L81" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="M81" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="N81" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="O81" s="2" t="s">
-        <v>422</v>
-      </c>
       <c r="P81" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q81" s="2" t="s">
         <v>31</v>
@@ -6843,11 +6823,11 @@
       <c r="U81" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="V81" s="3" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="82" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+      <c r="V81" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -6855,13 +6835,13 @@
         <v>22</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>50</v>
@@ -6870,26 +6850,26 @@
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K82" s="2"/>
       <c r="L82" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M82" s="2" t="s">
-        <v>568</v>
+        <v>556</v>
       </c>
       <c r="N82" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O82" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="P82" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q82" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O82" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="P82" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q82" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R82" s="2"/>
       <c r="S82" s="2" t="s">
@@ -6899,13 +6879,13 @@
         <v>40</v>
       </c>
       <c r="U82" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V82" s="2" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="83" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -6913,13 +6893,13 @@
         <v>22</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>50</v>
@@ -6928,26 +6908,26 @@
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
       <c r="J83" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K83" s="2"/>
       <c r="L83" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M83" s="2" t="s">
-        <v>569</v>
+        <v>557</v>
       </c>
       <c r="N83" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O83" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="P83" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q83" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O83" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="P83" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q83" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R83" s="2"/>
       <c r="S83" s="2" t="s">
@@ -6957,13 +6937,13 @@
         <v>40</v>
       </c>
       <c r="U83" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V83" s="2" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="84" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -6971,13 +6951,13 @@
         <v>22</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>50</v>
@@ -6986,26 +6966,26 @@
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K84" s="2"/>
       <c r="L84" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M84" s="2" t="s">
-        <v>572</v>
+        <v>560</v>
       </c>
       <c r="N84" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O84" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="P84" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q84" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O84" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="P84" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q84" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R84" s="2"/>
       <c r="S84" s="2" t="s">
@@ -7015,13 +6995,13 @@
         <v>40</v>
       </c>
       <c r="U84" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V84" s="2" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="85" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -7029,13 +7009,13 @@
         <v>22</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>50</v>
@@ -7044,26 +7024,26 @@
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
       <c r="J85" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K85" s="2"/>
       <c r="L85" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M85" s="2" t="s">
-        <v>573</v>
+        <v>561</v>
       </c>
       <c r="N85" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O85" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="P85" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q85" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O85" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="P85" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q85" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R85" s="2"/>
       <c r="S85" s="2" t="s">
@@ -7073,13 +7053,13 @@
         <v>40</v>
       </c>
       <c r="U85" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V85" s="2" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="86" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -7087,13 +7067,13 @@
         <v>22</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>50</v>
@@ -7102,14 +7082,14 @@
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K86" s="2"/>
       <c r="L86" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M86" s="2" t="s">
-        <v>589</v>
+        <v>577</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -7123,13 +7103,13 @@
         <v>40</v>
       </c>
       <c r="U86" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V86" s="2" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="87" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -7137,13 +7117,13 @@
         <v>22</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>50</v>
@@ -7152,14 +7132,14 @@
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K87" s="2"/>
       <c r="L87" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M87" s="2" t="s">
-        <v>591</v>
+        <v>579</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -7173,13 +7153,13 @@
         <v>40</v>
       </c>
       <c r="U87" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V87" s="2" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="88" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -7187,13 +7167,13 @@
         <v>22</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>50</v>
@@ -7202,14 +7182,14 @@
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K88" s="2"/>
       <c r="L88" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M88" s="2" t="s">
-        <v>593</v>
+        <v>581</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -7223,13 +7203,13 @@
         <v>40</v>
       </c>
       <c r="U88" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V88" s="2" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="89" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -7237,13 +7217,13 @@
         <v>22</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>50</v>
@@ -7252,26 +7232,26 @@
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
       <c r="J89" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K89" s="2"/>
       <c r="L89" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M89" s="2" t="s">
-        <v>576</v>
+        <v>564</v>
       </c>
       <c r="N89" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O89" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="P89" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q89" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O89" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="P89" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q89" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R89" s="2"/>
       <c r="S89" s="2" t="s">
@@ -7281,13 +7261,13 @@
         <v>40</v>
       </c>
       <c r="U89" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V89" s="2" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="90" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -7295,13 +7275,13 @@
         <v>22</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>50</v>
@@ -7310,26 +7290,26 @@
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
       <c r="J90" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K90" s="2"/>
       <c r="L90" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M90" s="2" t="s">
-        <v>577</v>
+        <v>565</v>
       </c>
       <c r="N90" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O90" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="P90" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q90" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O90" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="P90" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q90" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R90" s="2"/>
       <c r="S90" s="2" t="s">
@@ -7339,13 +7319,13 @@
         <v>40</v>
       </c>
       <c r="U90" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V90" s="2" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="91" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -7353,13 +7333,13 @@
         <v>22</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>50</v>
@@ -7368,26 +7348,26 @@
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
       <c r="J91" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K91" s="2"/>
       <c r="L91" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M91" s="2" t="s">
-        <v>578</v>
+        <v>566</v>
       </c>
       <c r="N91" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O91" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="P91" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q91" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O91" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="P91" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q91" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R91" s="2"/>
       <c r="S91" s="2" t="s">
@@ -7397,13 +7377,13 @@
         <v>40</v>
       </c>
       <c r="U91" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V91" s="2" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="92" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -7411,13 +7391,13 @@
         <v>22</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>50</v>
@@ -7426,26 +7406,26 @@
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K92" s="2"/>
       <c r="L92" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M92" s="2" t="s">
-        <v>579</v>
+        <v>567</v>
       </c>
       <c r="N92" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O92" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="P92" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q92" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O92" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="P92" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q92" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R92" s="2"/>
       <c r="S92" s="2" t="s">
@@ -7455,13 +7435,13 @@
         <v>40</v>
       </c>
       <c r="U92" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V92" s="2" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="93" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -7469,13 +7449,13 @@
         <v>22</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>50</v>
@@ -7484,11 +7464,11 @@
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K93" s="2"/>
       <c r="L93" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M93" s="2" t="s">
         <v>39</v>
@@ -7511,7 +7491,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="94" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -7519,13 +7499,13 @@
         <v>22</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>50</v>
@@ -7534,26 +7514,26 @@
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K94" s="2"/>
       <c r="L94" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M94" s="2" t="s">
-        <v>583</v>
+        <v>571</v>
       </c>
       <c r="N94" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O94" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="P94" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q94" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O94" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="P94" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q94" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R94" s="2"/>
       <c r="S94" s="2" t="s">
@@ -7563,13 +7543,13 @@
         <v>40</v>
       </c>
       <c r="U94" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V94" s="2" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="95" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -7577,13 +7557,13 @@
         <v>22</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>50</v>
@@ -7592,14 +7572,14 @@
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K95" s="2"/>
       <c r="L95" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M95" s="2" t="s">
-        <v>595</v>
+        <v>583</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -7613,13 +7593,13 @@
         <v>40</v>
       </c>
       <c r="U95" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V95" s="2" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="96" spans="1:22" ht="313.5" x14ac:dyDescent="0.25">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -7627,13 +7607,13 @@
         <v>22</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>50</v>
@@ -7642,11 +7622,11 @@
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K96" s="2"/>
       <c r="L96" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M96" s="2" t="s">
         <v>39</v>
@@ -7669,7 +7649,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -7677,13 +7657,13 @@
         <v>22</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>50</v>
@@ -7692,11 +7672,11 @@
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K97" s="2"/>
       <c r="L97" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M97" s="2" t="s">
         <v>39</v>
@@ -7719,7 +7699,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -7727,13 +7707,13 @@
         <v>22</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>50</v>
@@ -7742,11 +7722,11 @@
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K98" s="2"/>
       <c r="L98" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M98" s="2" t="s">
         <v>39</v>
@@ -7769,7 +7749,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -7777,13 +7757,13 @@
         <v>22</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>50</v>
@@ -7792,26 +7772,26 @@
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
       <c r="J99" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K99" s="2"/>
       <c r="L99" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M99" s="2" t="s">
-        <v>588</v>
+        <v>576</v>
       </c>
       <c r="N99" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O99" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="P99" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q99" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O99" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="P99" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q99" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R99" s="2"/>
       <c r="S99" s="2" t="s">
@@ -7821,13 +7801,13 @@
         <v>40</v>
       </c>
       <c r="U99" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V99" s="2" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="100" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -7835,13 +7815,13 @@
         <v>22</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>50</v>
@@ -7850,26 +7830,26 @@
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="K100" s="2"/>
       <c r="L100" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M100" s="2" t="s">
-        <v>587</v>
+        <v>575</v>
       </c>
       <c r="N100" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O100" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="P100" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q100" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="O100" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="P100" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="Q100" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="R100" s="2"/>
       <c r="S100" s="2" t="s">
@@ -7879,13 +7859,13 @@
         <v>40</v>
       </c>
       <c r="U100" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V100" s="2" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="101" spans="1:23" ht="327.75" x14ac:dyDescent="0.25">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -7893,13 +7873,13 @@
         <v>22</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>50</v>
@@ -7908,23 +7888,23 @@
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="K101" s="2"/>
       <c r="L101" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M101" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="O101" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="P101" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q101" s="2" t="s">
         <v>31</v>
@@ -7940,10 +7920,10 @@
         <v>68</v>
       </c>
       <c r="V101" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="102" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="102" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -7951,13 +7931,13 @@
         <v>22</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>50</v>
@@ -7966,23 +7946,23 @@
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="K102" s="2"/>
       <c r="L102" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M102" s="2" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="N102" s="2" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="O102" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="P102" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q102" s="2" t="s">
         <v>31</v>
@@ -7998,10 +7978,10 @@
         <v>68</v>
       </c>
       <c r="V102" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="103" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="103" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -8009,13 +7989,13 @@
         <v>22</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>50</v>
@@ -8024,23 +8004,23 @@
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
       <c r="J103" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="K103" s="2"/>
       <c r="L103" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M103" s="2" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="O103" s="2" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="P103" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="Q103" s="2" t="s">
         <v>31</v>
@@ -8056,10 +8036,10 @@
         <v>68</v>
       </c>
       <c r="V103" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="104" spans="1:23" ht="370.5" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" ht="313.5" x14ac:dyDescent="0.2">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -8067,13 +8047,13 @@
         <v>22</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>50</v>
@@ -8082,45 +8062,45 @@
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="K104" s="2"/>
       <c r="L104" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="M104" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N104" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="O104" s="3" t="s">
-        <v>560</v>
-      </c>
-      <c r="P104" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="Q104" s="3" t="s">
-        <v>397</v>
+      <c r="N104" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="O104" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="P104" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="Q104" s="2" t="s">
+        <v>394</v>
       </c>
       <c r="R104" s="2"/>
       <c r="S104" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="T104" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="U104" s="2" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="V104" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="W104" s="3" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="105" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+        <v>554</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="105" spans="1:23" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -8128,13 +8108,13 @@
         <v>22</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>50</v>
@@ -8143,26 +8123,26 @@
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
       <c r="J105" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="K105" s="2"/>
       <c r="L105" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="M105" s="3" t="s">
-        <v>564</v>
-      </c>
-      <c r="N105" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="O105" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="P105" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="Q105" s="3" t="s">
-        <v>561</v>
+        <v>319</v>
+      </c>
+      <c r="M105" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="N105" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="O105" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="P105" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q105" s="2" t="s">
+        <v>549</v>
       </c>
       <c r="R105" s="2"/>
       <c r="S105" s="2" t="s">
@@ -8171,14 +8151,14 @@
       <c r="T105" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="U105" s="3" t="s">
+      <c r="U105" s="2" t="s">
         <v>68</v>
       </c>
       <c r="V105" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="106" spans="1:23" ht="313.5" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="106" spans="1:23" ht="327.75" x14ac:dyDescent="0.2">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -8186,13 +8166,13 @@
         <v>22</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>50</v>
@@ -8201,25 +8181,25 @@
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="K106" s="2"/>
-      <c r="L106" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="M106" s="3" t="s">
-        <v>565</v>
-      </c>
-      <c r="N106" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="O106" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="P106" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="Q106" s="3" t="s">
+      <c r="L106" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M106" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="N106" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="O106" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="P106" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q106" s="2" t="s">
         <v>31</v>
       </c>
       <c r="R106" s="2"/>
@@ -8233,10 +8213,10 @@
         <v>68</v>
       </c>
       <c r="V106" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="107" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="107" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -8244,13 +8224,13 @@
         <v>22</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>50</v>
@@ -8259,7 +8239,7 @@
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="K107" s="2"/>
       <c r="L107" s="2"/>
@@ -8284,7 +8264,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -8292,13 +8272,13 @@
         <v>22</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>50</v>
@@ -8307,7 +8287,7 @@
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="K108" s="2"/>
       <c r="L108" s="2"/>
@@ -8332,7 +8312,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -8340,13 +8320,13 @@
         <v>22</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>50</v>
@@ -8355,7 +8335,7 @@
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
       <c r="J109" s="2" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="K109" s="2"/>
       <c r="L109" s="2"/>
@@ -8380,7 +8360,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -8388,13 +8368,13 @@
         <v>22</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>50</v>
@@ -8403,7 +8383,7 @@
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
       <c r="J110" s="2" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="K110" s="2"/>
       <c r="L110" s="2"/>
@@ -8428,7 +8408,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="99.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:23" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -8436,13 +8416,13 @@
         <v>22</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>50</v>
@@ -8451,10 +8431,10 @@
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
       <c r="J111" s="2" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="L111" s="2"/>
       <c r="M111" s="2" t="s">
@@ -8478,7 +8458,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:23" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -8486,13 +8466,13 @@
         <v>22</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>50</v>
@@ -8501,7 +8481,7 @@
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="K112" s="2"/>
       <c r="L112" s="2"/>
@@ -8526,7 +8506,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="113" spans="1:22" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:22" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -8534,13 +8514,13 @@
         <v>22</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>50</v>
@@ -8549,7 +8529,7 @@
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="K113" s="2"/>
       <c r="L113" s="2"/>
@@ -8574,194 +8554,8 @@
         <v>86</v>
       </c>
     </row>
-    <row r="114" spans="1:22" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A114" s="2">
-        <v>113</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>542</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G114" s="2"/>
-      <c r="H114" s="2"/>
-      <c r="I114" s="2"/>
-      <c r="J114" s="2"/>
-      <c r="K114" s="2"/>
-      <c r="L114" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="M114" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N114" s="2"/>
-      <c r="O114" s="2"/>
-      <c r="P114" s="2"/>
-      <c r="Q114" s="2"/>
-      <c r="R114" s="2"/>
-      <c r="S114" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="T114" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="U114" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="V114" s="2" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A115" s="2">
-        <v>114</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="F115" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G115" s="2"/>
-      <c r="H115" s="2"/>
-      <c r="I115" s="2"/>
-      <c r="J115" s="2"/>
-      <c r="K115" s="2"/>
-      <c r="L115" s="2"/>
-      <c r="M115" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N115" s="2"/>
-      <c r="O115" s="2"/>
-      <c r="P115" s="2"/>
-      <c r="Q115" s="2"/>
-      <c r="R115" s="2"/>
-      <c r="S115" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T115" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="U115" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="V115" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A116" s="2">
-        <v>115</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G116" s="2"/>
-      <c r="H116" s="2"/>
-      <c r="I116" s="2"/>
-      <c r="J116" s="2"/>
-      <c r="K116" s="2"/>
-      <c r="L116" s="2"/>
-      <c r="M116" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N116" s="2"/>
-      <c r="O116" s="2"/>
-      <c r="P116" s="2"/>
-      <c r="Q116" s="2"/>
-      <c r="R116" s="2"/>
-      <c r="S116" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T116" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="U116" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="V116" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A117" s="2">
-        <v>116</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>549</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="F117" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G117" s="2"/>
-      <c r="H117" s="2"/>
-      <c r="I117" s="2"/>
-      <c r="J117" s="2"/>
-      <c r="K117" s="2"/>
-      <c r="L117" s="2"/>
-      <c r="M117" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N117" s="2"/>
-      <c r="O117" s="2"/>
-      <c r="P117" s="2"/>
-      <c r="Q117" s="2"/>
-      <c r="R117" s="2"/>
-      <c r="S117" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T117" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="U117" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="V117" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V117" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V113" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>